<commit_message>
spec-339336224: 17 позиций, ИТОГО 2 649 287,08 ₽
</commit_message>
<xml_diff>
--- a/vse-loti/339336224/spec-339336224.xlsx
+++ b/vse-loti/339336224/spec-339336224.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -497,19 +497,644 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ТРУБА 76Х3.5 СТ20 ГОСТ10704</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>4.276</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>4.276</v>
+      </c>
+      <c r="F2" t="n">
+        <v>49487.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>59385</v>
+      </c>
+      <c r="H2" t="n">
+        <v>211608.55</v>
+      </c>
+      <c r="I2" t="n">
+        <v>49487.5</v>
+      </c>
+      <c r="J2" t="n">
+        <v>59385</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ТРУБА 820Х10 СТ17Г1С ТИП3 К52 ГОСТ20295</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2.397</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2.397</v>
+      </c>
+      <c r="F3" t="n">
+        <v>64107.62</v>
+      </c>
+      <c r="G3" t="n">
+        <v>76929.14</v>
+      </c>
+      <c r="H3" t="n">
+        <v>153665.97</v>
+      </c>
+      <c r="I3" t="n">
+        <v>64107.62</v>
+      </c>
+      <c r="J3" t="n">
+        <v>76929.14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ТРУБА 32Х3.2 СТ3СП ГОСТ3262</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="F4" t="n">
+        <v>51009.2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>61211.04</v>
+      </c>
+      <c r="H4" t="n">
+        <v>8518.540000000001</v>
+      </c>
+      <c r="I4" t="n">
+        <v>51009.2</v>
+      </c>
+      <c r="J4" t="n">
+        <v>61211.04</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ТРУБА 108Х5 СТ20 ГОСТ10704</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.529</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.529</v>
+      </c>
+      <c r="F5" t="n">
+        <v>105482.77</v>
+      </c>
+      <c r="G5" t="n">
+        <v>126579.32</v>
+      </c>
+      <c r="H5" t="n">
+        <v>55800.39</v>
+      </c>
+      <c r="I5" t="n">
+        <v>105482.77</v>
+      </c>
+      <c r="J5" t="n">
+        <v>126579.32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ТРУБА 133Х4 СТ20 ГОСТ10704</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="F6" t="n">
+        <v>62724.47</v>
+      </c>
+      <c r="G6" t="n">
+        <v>75269.36</v>
+      </c>
+      <c r="H6" t="n">
+        <v>57518.34</v>
+      </c>
+      <c r="I6" t="n">
+        <v>62724.47</v>
+      </c>
+      <c r="J6" t="n">
+        <v>75269.36</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ТРУБА 159Х4.5 СТ20 ГОСТ10704</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F7" t="n">
+        <v>99150</v>
+      </c>
+      <c r="G7" t="n">
+        <v>118980</v>
+      </c>
+      <c r="H7" t="n">
+        <v>23796</v>
+      </c>
+      <c r="I7" t="n">
+        <v>99150</v>
+      </c>
+      <c r="J7" t="n">
+        <v>118980</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ТРУБА 89Х3.5 СТ20 ГОСТ10704</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4.959</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>4.959</v>
+      </c>
+      <c r="F8" t="n">
+        <v>70819.23</v>
+      </c>
+      <c r="G8" t="n">
+        <v>84983.08</v>
+      </c>
+      <c r="H8" t="n">
+        <v>351192.56</v>
+      </c>
+      <c r="I8" t="n">
+        <v>70819.23</v>
+      </c>
+      <c r="J8" t="n">
+        <v>84983.08</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ТРУБА 57Х3.5 СТ3СП ГОСТ10705</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2.809</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2.809</v>
+      </c>
+      <c r="F9" t="n">
+        <v>89880</v>
+      </c>
+      <c r="G9" t="n">
+        <v>107856</v>
+      </c>
+      <c r="H9" t="n">
+        <v>252472.92</v>
+      </c>
+      <c r="I9" t="n">
+        <v>89880</v>
+      </c>
+      <c r="J9" t="n">
+        <v>107856</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ТРУБА 325Х8 СТ20 ГОСТ10704</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4.503</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>4.503</v>
+      </c>
+      <c r="F10" t="n">
+        <v>57066.66</v>
+      </c>
+      <c r="G10" t="n">
+        <v>68479.99000000001</v>
+      </c>
+      <c r="H10" t="n">
+        <v>256971.17</v>
+      </c>
+      <c r="I10" t="n">
+        <v>57066.66</v>
+      </c>
+      <c r="J10" t="n">
+        <v>68479.99000000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ТРУБА 20Х2.8 СТ2ПС ГОСТ3262</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="n">
+        <v>76847.39999999999</v>
+      </c>
+      <c r="G11" t="n">
+        <v>92216.88</v>
+      </c>
+      <c r="H11" t="n">
+        <v>307389.6</v>
+      </c>
+      <c r="I11" t="n">
+        <v>76847.39999999999</v>
+      </c>
+      <c r="J11" t="n">
+        <v>92216.88</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ТРУБА 630Х8 СТ20 ГОСТ10704</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>4.418</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>4.418</v>
+      </c>
+      <c r="F12" t="n">
+        <v>117293.4</v>
+      </c>
+      <c r="G12" t="n">
+        <v>140752.08</v>
+      </c>
+      <c r="H12" t="n">
+        <v>518202.24</v>
+      </c>
+      <c r="I12" t="n">
+        <v>117293.4</v>
+      </c>
+      <c r="J12" t="n">
+        <v>140752.08</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ТРУБА 25Х3.2 СТ3СП ГОСТ3262</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F13" t="n">
+        <v>68758.2</v>
+      </c>
+      <c r="G13" t="n">
+        <v>82509.84</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1856.47</v>
+      </c>
+      <c r="I13" t="n">
+        <v>68758.2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>82509.84</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ТРУБА 273Х8 СТ10 ГОСТ10704</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.541</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0.541</v>
+      </c>
+      <c r="F14" t="n">
+        <v>79680.17</v>
+      </c>
+      <c r="G14" t="n">
+        <v>95616.2</v>
+      </c>
+      <c r="H14" t="n">
+        <v>43106.97</v>
+      </c>
+      <c r="I14" t="n">
+        <v>79680.17</v>
+      </c>
+      <c r="J14" t="n">
+        <v>95616.2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ТРУБА 219Х6 СТ20 ГОСТ10704</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4.918</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>4.918</v>
+      </c>
+      <c r="F15" t="n">
+        <v>63237</v>
+      </c>
+      <c r="G15" t="n">
+        <v>75884.39999999999</v>
+      </c>
+      <c r="H15" t="n">
+        <v>310999.57</v>
+      </c>
+      <c r="I15" t="n">
+        <v>63237</v>
+      </c>
+      <c r="J15" t="n">
+        <v>75884.39999999999</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ТРУБА 108Х4.0 СТ20 ОЦИНК. ГОСТ10705</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="F16" t="n">
+        <v>85600</v>
+      </c>
+      <c r="G16" t="n">
+        <v>102720</v>
+      </c>
+      <c r="H16" t="n">
+        <v>14124</v>
+      </c>
+      <c r="I16" t="n">
+        <v>85600</v>
+      </c>
+      <c r="J16" t="n">
+        <v>102720</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ТРУБА 377Х8 СТ20 ГОСТ10704</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.874</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0.874</v>
+      </c>
+      <c r="F17" t="n">
+        <v>55833.29</v>
+      </c>
+      <c r="G17" t="n">
+        <v>66999.95</v>
+      </c>
+      <c r="H17" t="n">
+        <v>48798.3</v>
+      </c>
+      <c r="I17" t="n">
+        <v>55833.29</v>
+      </c>
+      <c r="J17" t="n">
+        <v>66999.95</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ТРУБА 80Х4 СТ20 ГОСТ3262</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="F18" t="n">
+        <v>113922.9</v>
+      </c>
+      <c r="G18" t="n">
+        <v>136707.48</v>
+      </c>
+      <c r="H18" t="n">
+        <v>33265.49</v>
+      </c>
+      <c r="I18" t="n">
+        <v>113922.9</v>
+      </c>
+      <c r="J18" t="n">
+        <v>136707.48</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Источник: Обоснование НМЦ.docx.DOCX</t>
+      <c r="E19" s="2" t="n">
+        <v>36.032</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>2649287.08</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>НМЦК из обоснования:</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>2649287.08</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Источник: ВЛТС_ЭТЗ на децентрализованную поставку труб стальных для ВлТС в 2027 г_.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>